<commit_message>
feat: adjustments to scripts, column titles and updating of datasets
</commit_message>
<xml_diff>
--- a/metadata/old/extract_v2/diet/SDDs/SDD-NHANES-1999-2000-DSQFILE1.xlsx
+++ b/metadata/old/extract_v2/diet/SDDs/SDD-NHANES-1999-2000-DSQFILE1.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t>Column</t>
   </si>
@@ -26,6 +26,63 @@
     <t>Label</t>
   </si>
   <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Other For</t>
+  </si>
+  <si>
+    <t>SEQN</t>
+  </si>
+  <si>
+    <t>DSD010</t>
+  </si>
+  <si>
+    <t>DSDCOUNT</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>0 To 20</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>99</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Refused</t>
+  </si>
+  <si>
+    <t>Don'T Know</t>
+  </si>
+  <si>
+    <t>Missing</t>
+  </si>
+  <si>
+    <t>Range Of Values</t>
+  </si>
+  <si>
     <t>English_Text</t>
   </si>
   <si>
@@ -35,61 +92,40 @@
     <t>English_Instructions</t>
   </si>
   <si>
-    <t>Class</t>
-  </si>
-  <si>
-    <t>Other For</t>
-  </si>
-  <si>
-    <t>SEQN</t>
-  </si>
-  <si>
-    <t>DSD010</t>
-  </si>
-  <si>
-    <t>DSDCOUNT</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>.</t>
-  </si>
-  <si>
-    <t>0 To 20</t>
-  </si>
-  <si>
-    <t>77</t>
-  </si>
-  <si>
-    <t>99</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Refused</t>
-  </si>
-  <si>
-    <t>Don'T Know</t>
-  </si>
-  <si>
-    <t>Missing</t>
-  </si>
-  <si>
-    <t>Range Of Values</t>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>attributeOf</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Entity</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Relation</t>
+  </si>
+  <si>
+    <t>inRelationTo</t>
+  </si>
+  <si>
+    <t>wasDerivedFrom</t>
+  </si>
+  <si>
+    <t>Maturity</t>
+  </si>
+  <si>
+    <t>Template</t>
+  </si>
+  <si>
+    <t>wasGeneratedBy</t>
   </si>
   <si>
     <t>Respondent sequence number.</t>
@@ -102,45 +138,6 @@
   </si>
   <si>
     <t>Both males and females 0 YEARS - 150 YEARS</t>
-  </si>
-  <si>
-    <t>nan</t>
-  </si>
-  <si>
-    <t>Attribute</t>
-  </si>
-  <si>
-    <t>attributeOf</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Entity</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Relation</t>
-  </si>
-  <si>
-    <t>inRelationTo</t>
-  </si>
-  <si>
-    <t>wasDerivedFrom</t>
-  </si>
-  <si>
-    <t>Maturity</t>
-  </si>
-  <si>
-    <t>Template</t>
-  </si>
-  <si>
-    <t>wasGeneratedBy</t>
   </si>
 </sst>
 </file>
@@ -498,10 +495,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,208 +514,109 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C11" t="s">
         <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" t="s">
-        <v>28</v>
-      </c>
-      <c r="F9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" t="s">
-        <v>28</v>
-      </c>
-      <c r="F10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -728,63 +626,90 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
         <v>39</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="C4" t="s">
         <v>40</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>